<commit_message>
배포판 자동 동기화 — a82858a (claude/python-program-2ugsof)
비공개 저장소의 소스에서 py_app.zip을 새로 굽고 배포 파일을 맞췄습니다.
이 커밋은 GitHub Actions가 자동으로 만든 것입니다.
</commit_message>
<xml_diff>
--- a/templates/입력2_연간근무표_2026-08.xlsx
+++ b/templates/입력2_연간근무표_2026-08.xlsx
@@ -557,14 +557,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>입력③ 연간근무표 — 양식 안내</t>
+          <t>입력② 연간근무표 — 양식 안내</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>다월 자동 연동용 파일입니다. 지난달 생성 후 받은 '연간근무표'를 그대로 다시 올리면, 인원 명단·누적 통계(야간·근무일·OFF 등 형평성 지표)뿐 아니라 전월이월값(마지막 근무·연속근무일수·야간블록 등)까지 이번 달 생성에 자동으로 이어집니다 — 예전의 '입력③ 월간근무표(전월)'을 따로 올릴 필요가 없어졌습니다.</t>
+          <t>다월 자동 연동용 파일입니다. 지난달 생성 후 받은 '연간근무표'(출력②)를 그대로 다시 올리면, 인원 명단·누적 통계(야간·근무일·OFF 등 형평성 지표)뿐 아니라 전월이월값(마지막 근무·연속근무일수·야간블록 등)까지 이번 달 생성에 자동으로 이어집니다 — 지난달 월간근무표를 따로 올릴 필요가 없습니다.</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>· 인원 정보 — 순번·이름·직급·숙련도·가능근무·비고·전입·전입일. 파트장이 맨 위, 나머지는 입력①에 등록된 순서 그대로 나열됩니다.</t>
+          <t>· 인원 정보 — 순번·이름·직급·숙련도·가능근무·비고·전입·전입일. 파트장이 맨 위, 나머지는 입력①(원티드표)에 등록된 순서 그대로 나열됩니다.</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>① 기존 인원 목록 바로 아래(맨 아래 '레벨평균' 줄보다 위)에 행을 추가하고 이름·직급·숙련도·가능근무를 적습니다. 이름은 입력②(원티드표)와 정확히 같아야 합니다.</t>
+          <t>① 기존 인원 목록 바로 아래(맨 아래 'D 인원'~'Lv1-3' 통계 줄보다 위)에 행을 추가하고 이름·직급·숙련도·가능근무를 적습니다. 이름은 입력①(원티드표)과 정확히 같아야 합니다.</t>
         </is>
       </c>
     </row>
@@ -662,7 +662,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>따로 적으실 게 없습니다. 입력②(이번 달 명단)에 없으면 자동으로 전출로 보고 이번 달 배정에서 빼며, 그동안 쌓인 이력은 아래쪽 '전출' 구분 행 밑에 그대로 보존됩니다.</t>
+          <t>따로 적으실 게 없습니다. 입력①(원티드표, 이번 달 명단)에 없으면 자동으로 전출로 보고 이번 달 배정에서 빼며, 그동안 쌓인 이력은 아래쪽 '전출' 구분 행 밑에 그대로 보존됩니다.</t>
         </is>
       </c>
     </row>
@@ -676,11 +676,10 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>이 파일 없이 생략해도 됩니다 — 입력①②만으로 근무표 생성이 가능하고, 이 앱이 매달 자동으로 연간근무표를 만들어 드리니 다음 달부터 이어받으면 됩니다.</t>
+          <t>이 파일 없이 생략해도 됩니다 — 입력①(원티드표)만으로 근무표 생성이 가능하고, 이 앱이 매달 자동으로 연간근무표를 만들어 드리니 다음 달부터 이어받으면 됩니다.</t>
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
@@ -16584,7 +16583,6 @@
         </is>
       </c>
     </row>
-    <row r="45"/>
     <row r="46">
       <c r="B46" s="20" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
배포판 자동 동기화 — 6443dd1 (claude/python-program-2ugsof)
비공개 저장소의 소스에서 py_app.zip을 새로 굽고 배포 파일을 맞췄습니다.
이 커밋은 GitHub Actions가 자동으로 만든 것입니다.
</commit_message>
<xml_diff>
--- a/templates/입력2_연간근무표_2026-08.xlsx
+++ b/templates/입력2_연간근무표_2026-08.xlsx
@@ -869,12 +869,12 @@
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>누적2일블록</t>
+          <t>누적 2일 블록 야간</t>
         </is>
       </c>
       <c r="N3" s="4" t="inlineStr">
         <is>
-          <t>누적3일블록</t>
+          <t>누적 3일 블록 야간</t>
         </is>
       </c>
       <c r="O3" s="4" t="inlineStr">
@@ -904,7 +904,7 @@
       </c>
       <c r="T3" s="4" t="inlineStr">
         <is>
-          <t>누적주말휴일오프</t>
+          <t>누적주말휴일오프_total(설,추석 포함)</t>
         </is>
       </c>
       <c r="U3" s="4" t="inlineStr">
@@ -16717,7 +16717,6 @@
         </is>
       </c>
     </row>
-    <row r="45"/>
     <row r="46">
       <c r="B46" s="20" t="inlineStr">
         <is>

</xml_diff>